<commit_message>
Removing the "PCR Due" column
</commit_message>
<xml_diff>
--- a/core/api/export/templates/APRAnnexI.xlsx
+++ b/core/api/export/templates/APRAnnexI.xlsx
@@ -16,7 +16,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment authorId="0" ref="AU1">
+    <comment authorId="0" ref="AT1">
       <text>
         <t xml:space="preserve">XX meeting, based on the year of the APR and the last ExCom meeting held before the APR. to be derived
 	-Rony Salim Aoun</t>
@@ -27,10 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="60">
-  <si>
-    <t>PCR Due</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>Meta Code</t>
   </si>
@@ -182,9 +179,6 @@
     <t>Gender Policy for All Projects Approved from 85th Mtg (Yes/No)</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>IVC/ARS/46/INV/23</t>
   </si>
   <si>
@@ -207,6 +201,9 @@
   </si>
   <si>
     <t>CLO</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -336,7 +333,6 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
@@ -361,6 +357,7 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -581,28 +578,28 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0" outlineLevelCol="1"/>
   <cols>
-    <col customWidth="1" min="1" max="2" width="10.75"/>
-    <col customWidth="1" min="3" max="4" width="11.25"/>
-    <col customWidth="1" min="5" max="10" width="9.25"/>
-    <col customWidth="1" min="11" max="11" width="26.5"/>
-    <col customWidth="1" min="12" max="12" width="9.25"/>
-    <col customWidth="1" min="13" max="13" width="11.13"/>
-    <col customWidth="1" min="14" max="18" width="10.13" outlineLevel="1"/>
-    <col customWidth="1" min="19" max="24" width="9.25"/>
-    <col customWidth="1" min="25" max="30" width="11.13" outlineLevel="1"/>
-    <col customWidth="1" min="31" max="36" width="9.25"/>
-    <col customWidth="1" min="37" max="37" width="12.75"/>
-    <col customWidth="1" min="38" max="38" width="12.88"/>
-    <col customWidth="1" min="39" max="39" width="11.25"/>
-    <col customWidth="1" min="40" max="44" width="9.25" outlineLevel="1"/>
-    <col customWidth="1" min="45" max="46" width="12.13" outlineLevel="1"/>
-    <col customWidth="1" min="47" max="47" width="13.13"/>
-    <col customWidth="1" min="48" max="48" width="12.13"/>
-    <col customWidth="1" min="49" max="51" width="21.38" outlineLevel="1"/>
-    <col customWidth="1" min="52" max="52" width="10.63"/>
-    <col customWidth="1" min="53" max="55" width="9.25"/>
-    <col customWidth="1" min="56" max="57" width="12.25"/>
-    <col customWidth="1" min="58" max="58" width="9.25"/>
+    <col customWidth="1" min="1" max="1" width="10.75"/>
+    <col customWidth="1" min="2" max="3" width="11.25"/>
+    <col customWidth="1" min="4" max="9" width="9.25"/>
+    <col customWidth="1" min="10" max="10" width="26.5"/>
+    <col customWidth="1" min="11" max="11" width="9.25"/>
+    <col customWidth="1" min="12" max="12" width="11.13"/>
+    <col customWidth="1" min="13" max="17" width="10.13" outlineLevel="1"/>
+    <col customWidth="1" min="18" max="23" width="9.25"/>
+    <col customWidth="1" min="24" max="29" width="11.13" outlineLevel="1"/>
+    <col customWidth="1" min="30" max="35" width="9.25"/>
+    <col customWidth="1" min="36" max="36" width="12.75"/>
+    <col customWidth="1" min="37" max="37" width="12.88"/>
+    <col customWidth="1" min="38" max="38" width="11.25"/>
+    <col customWidth="1" min="39" max="43" width="9.25" outlineLevel="1"/>
+    <col customWidth="1" min="44" max="45" width="12.13" outlineLevel="1"/>
+    <col customWidth="1" min="46" max="46" width="13.13"/>
+    <col customWidth="1" min="47" max="47" width="12.13"/>
+    <col customWidth="1" min="48" max="50" width="21.38" outlineLevel="1"/>
+    <col customWidth="1" min="51" max="51" width="10.63"/>
+    <col customWidth="1" min="52" max="54" width="9.25"/>
+    <col customWidth="1" min="55" max="56" width="12.25"/>
+    <col customWidth="1" min="57" max="57" width="9.25"/>
   </cols>
   <sheetData>
     <row r="1" ht="99.75" customHeight="1">
@@ -642,7 +639,7 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="2" t="s">
@@ -657,7 +654,7 @@
       <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="1" t="s">
@@ -675,7 +672,7 @@
       <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
       <c r="Y1" s="2" t="s">
@@ -693,7 +690,7 @@
       <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
       <c r="AE1" s="1" t="s">
@@ -702,10 +699,10 @@
       <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AG1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="3" t="s">
+      <c r="AH1" s="1" t="s">
         <v>33</v>
       </c>
       <c r="AI1" s="1" t="s">
@@ -720,7 +717,7 @@
       <c r="AL1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AM1" s="2" t="s">
         <v>38</v>
       </c>
       <c r="AN1" s="2" t="s">
@@ -735,187 +732,181 @@
       <c r="AQ1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AR1" s="4" t="s">
         <v>43</v>
       </c>
       <c r="AS1" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" s="4" t="s">
+      <c r="AT1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" s="5" t="s">
+      <c r="AU1" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" s="6" t="s">
+      <c r="AV1" s="7" t="s">
         <v>47</v>
       </c>
       <c r="AW1" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" s="7" t="s">
+      <c r="AX1" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AZ1" s="9"/>
+      <c r="AY1" s="9"/>
+      <c r="AZ1" s="10"/>
       <c r="BA1" s="10"/>
       <c r="BB1" s="10"/>
       <c r="BC1" s="10"/>
       <c r="BD1" s="10"/>
       <c r="BE1" s="10"/>
-      <c r="BF1" s="10"/>
     </row>
     <row r="2" ht="12.75" customHeight="1">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="13"/>
+      <c r="F2" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="G2" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="H2" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="I2" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="J2" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="K2" s="15">
+        <v>38534.0</v>
+      </c>
+      <c r="L2" s="15">
+        <v>39326.0</v>
+      </c>
+      <c r="M2" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="K2" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="L2" s="16">
-        <v>38534.0</v>
-      </c>
-      <c r="M2" s="16">
-        <v>39326.0</v>
-      </c>
-      <c r="N2" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="O2" s="16">
+      <c r="N2" s="15">
         <v>38626.0</v>
       </c>
-      <c r="P2" s="16">
+      <c r="O2" s="15">
         <v>38626.0</v>
       </c>
-      <c r="Q2" s="16">
+      <c r="P2" s="15">
         <v>38626.0</v>
       </c>
-      <c r="R2" s="16">
+      <c r="Q2" s="15">
         <v>39965.0</v>
       </c>
-      <c r="S2" s="17">
+      <c r="R2" s="16">
         <v>43.4</v>
       </c>
-      <c r="T2" s="17">
+      <c r="S2" s="16">
         <v>43.4</v>
       </c>
-      <c r="U2" s="17">
+      <c r="T2" s="16">
         <v>0.0</v>
       </c>
-      <c r="V2" s="17">
+      <c r="U2" s="16">
         <v>0.0</v>
       </c>
-      <c r="W2" s="17">
+      <c r="V2" s="16">
         <v>0.0</v>
       </c>
-      <c r="X2" s="17">
+      <c r="W2" s="16">
         <v>0.0</v>
       </c>
-      <c r="Y2" s="17">
+      <c r="X2" s="16">
         <v>0.0</v>
       </c>
-      <c r="Z2" s="17">
+      <c r="Y2" s="16">
         <v>0.0</v>
       </c>
-      <c r="AA2" s="17">
+      <c r="Z2" s="16">
         <v>0.0</v>
       </c>
-      <c r="AB2" s="17">
+      <c r="AA2" s="16">
         <v>0.0</v>
       </c>
-      <c r="AC2" s="17">
+      <c r="AB2" s="16">
+        <v>0.0</v>
+      </c>
+      <c r="AC2" s="16">
         <v>0.0</v>
       </c>
       <c r="AD2" s="17">
-        <v>0.0</v>
-      </c>
-      <c r="AE2" s="18">
         <v>110428.0</v>
       </c>
-      <c r="AF2" s="18">
+      <c r="AE2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AG2" s="18">
+      <c r="AF2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AH2" s="18">
+      <c r="AG2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AI2" s="18">
+      <c r="AH2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AJ2" s="18">
+      <c r="AI2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AK2" s="18">
+      <c r="AJ2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AL2" s="18">
+      <c r="AK2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AM2" s="18">
+      <c r="AL2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AN2" s="18">
+      <c r="AM2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AO2" s="18">
+      <c r="AN2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AP2" s="18">
+      <c r="AO2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AQ2" s="18">
+      <c r="AP2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AR2" s="18">
+      <c r="AQ2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AS2" s="18">
+      <c r="AR2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AT2" s="18">
+      <c r="AS2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AU2" s="19"/>
-      <c r="AV2" s="16">
+      <c r="AT2" s="18"/>
+      <c r="AU2" s="15">
         <v>39965.0</v>
       </c>
-      <c r="AW2" s="19"/>
-      <c r="AX2" s="19"/>
-      <c r="AY2" s="11" t="s">
-        <v>51</v>
+      <c r="AV2" s="18"/>
+      <c r="AW2" s="18"/>
+      <c r="AX2" s="19" t="s">
+        <v>58</v>
       </c>
-      <c r="AZ2" s="19"/>
-      <c r="BA2" s="19"/>
-      <c r="BB2" s="19"/>
-      <c r="BC2" s="19"/>
-      <c r="BD2" s="19"/>
-      <c r="BE2" s="19"/>
-      <c r="BF2" s="19"/>
+      <c r="AY2" s="18"/>
+      <c r="AZ2" s="18"/>
+      <c r="BA2" s="18"/>
+      <c r="BB2" s="18"/>
+      <c r="BC2" s="18"/>
+      <c r="BD2" s="18"/>
+      <c r="BE2" s="18"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="20"/>
@@ -935,8 +926,8 @@
       <c r="O3" s="20"/>
       <c r="P3" s="20"/>
       <c r="Q3" s="20"/>
-      <c r="R3" s="20"/>
-      <c r="S3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="20"/>
       <c r="T3" s="20"/>
       <c r="U3" s="20"/>
       <c r="V3" s="20"/>
@@ -975,7 +966,6 @@
       <c r="BC3" s="20"/>
       <c r="BD3" s="20"/>
       <c r="BE3" s="20"/>
-      <c r="BF3" s="20"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="20"/>
@@ -1035,7 +1025,6 @@
       <c r="BC4" s="20"/>
       <c r="BD4" s="20"/>
       <c r="BE4" s="20"/>
-      <c r="BF4" s="20"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="20"/>
@@ -1095,7 +1084,6 @@
       <c r="BC5" s="20"/>
       <c r="BD5" s="20"/>
       <c r="BE5" s="20"/>
-      <c r="BF5" s="20"/>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="20"/>
@@ -1155,7 +1143,6 @@
       <c r="BC6" s="20"/>
       <c r="BD6" s="20"/>
       <c r="BE6" s="20"/>
-      <c r="BF6" s="20"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="20"/>
@@ -1215,7 +1202,6 @@
       <c r="BC7" s="20"/>
       <c r="BD7" s="20"/>
       <c r="BE7" s="20"/>
-      <c r="BF7" s="20"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="20"/>
@@ -1275,7 +1261,6 @@
       <c r="BC8" s="20"/>
       <c r="BD8" s="20"/>
       <c r="BE8" s="20"/>
-      <c r="BF8" s="20"/>
     </row>
     <row r="9" ht="12.75" customHeight="1">
       <c r="A9" s="20"/>
@@ -1335,7 +1320,6 @@
       <c r="BC9" s="20"/>
       <c r="BD9" s="20"/>
       <c r="BE9" s="20"/>
-      <c r="BF9" s="20"/>
     </row>
     <row r="10" ht="12.75" customHeight="1">
       <c r="A10" s="20"/>
@@ -1395,7 +1379,6 @@
       <c r="BC10" s="20"/>
       <c r="BD10" s="20"/>
       <c r="BE10" s="20"/>
-      <c r="BF10" s="20"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="20"/>
@@ -1455,7 +1438,6 @@
       <c r="BC11" s="20"/>
       <c r="BD11" s="20"/>
       <c r="BE11" s="20"/>
-      <c r="BF11" s="20"/>
     </row>
     <row r="12" ht="12.75" customHeight="1">
       <c r="A12" s="20"/>
@@ -1515,7 +1497,6 @@
       <c r="BC12" s="20"/>
       <c r="BD12" s="20"/>
       <c r="BE12" s="20"/>
-      <c r="BF12" s="20"/>
     </row>
     <row r="13" ht="12.75" customHeight="1">
       <c r="A13" s="20"/>
@@ -1575,7 +1556,6 @@
       <c r="BC13" s="20"/>
       <c r="BD13" s="20"/>
       <c r="BE13" s="20"/>
-      <c r="BF13" s="20"/>
     </row>
     <row r="14" ht="12.75" customHeight="1">
       <c r="A14" s="20"/>
@@ -1635,7 +1615,6 @@
       <c r="BC14" s="20"/>
       <c r="BD14" s="20"/>
       <c r="BE14" s="20"/>
-      <c r="BF14" s="20"/>
     </row>
     <row r="15" ht="12.75" customHeight="1">
       <c r="A15" s="20"/>
@@ -1695,7 +1674,6 @@
       <c r="BC15" s="20"/>
       <c r="BD15" s="20"/>
       <c r="BE15" s="20"/>
-      <c r="BF15" s="20"/>
     </row>
     <row r="16" ht="12.75" customHeight="1">
       <c r="A16" s="20"/>
@@ -1755,7 +1733,6 @@
       <c r="BC16" s="20"/>
       <c r="BD16" s="20"/>
       <c r="BE16" s="20"/>
-      <c r="BF16" s="20"/>
     </row>
     <row r="17" ht="12.75" customHeight="1">
       <c r="A17" s="20"/>
@@ -1815,7 +1792,6 @@
       <c r="BC17" s="20"/>
       <c r="BD17" s="20"/>
       <c r="BE17" s="20"/>
-      <c r="BF17" s="20"/>
     </row>
     <row r="18" ht="12.75" customHeight="1">
       <c r="A18" s="20"/>
@@ -1875,7 +1851,6 @@
       <c r="BC18" s="20"/>
       <c r="BD18" s="20"/>
       <c r="BE18" s="20"/>
-      <c r="BF18" s="20"/>
     </row>
     <row r="19" ht="12.75" customHeight="1">
       <c r="A19" s="20"/>
@@ -1935,7 +1910,6 @@
       <c r="BC19" s="20"/>
       <c r="BD19" s="20"/>
       <c r="BE19" s="20"/>
-      <c r="BF19" s="20"/>
     </row>
     <row r="20" ht="12.75" customHeight="1">
       <c r="A20" s="20"/>
@@ -1995,7 +1969,6 @@
       <c r="BC20" s="20"/>
       <c r="BD20" s="20"/>
       <c r="BE20" s="20"/>
-      <c r="BF20" s="20"/>
     </row>
     <row r="21" ht="12.75" customHeight="1">
       <c r="A21" s="20"/>
@@ -2055,7 +2028,6 @@
       <c r="BC21" s="20"/>
       <c r="BD21" s="20"/>
       <c r="BE21" s="20"/>
-      <c r="BF21" s="20"/>
     </row>
     <row r="22" ht="12.75" customHeight="1">
       <c r="A22" s="20"/>
@@ -2115,7 +2087,6 @@
       <c r="BC22" s="20"/>
       <c r="BD22" s="20"/>
       <c r="BE22" s="20"/>
-      <c r="BF22" s="20"/>
     </row>
     <row r="23" ht="12.75" customHeight="1">
       <c r="A23" s="20"/>
@@ -2175,7 +2146,6 @@
       <c r="BC23" s="20"/>
       <c r="BD23" s="20"/>
       <c r="BE23" s="20"/>
-      <c r="BF23" s="20"/>
     </row>
     <row r="24" ht="12.75" customHeight="1">
       <c r="A24" s="20"/>
@@ -2235,7 +2205,6 @@
       <c r="BC24" s="20"/>
       <c r="BD24" s="20"/>
       <c r="BE24" s="20"/>
-      <c r="BF24" s="20"/>
     </row>
     <row r="25" ht="12.75" customHeight="1">
       <c r="A25" s="20"/>
@@ -2295,7 +2264,6 @@
       <c r="BC25" s="20"/>
       <c r="BD25" s="20"/>
       <c r="BE25" s="20"/>
-      <c r="BF25" s="20"/>
     </row>
     <row r="26" ht="12.75" customHeight="1">
       <c r="A26" s="20"/>
@@ -2355,7 +2323,6 @@
       <c r="BC26" s="20"/>
       <c r="BD26" s="20"/>
       <c r="BE26" s="20"/>
-      <c r="BF26" s="20"/>
     </row>
     <row r="27" ht="12.75" customHeight="1">
       <c r="A27" s="20"/>
@@ -2415,7 +2382,6 @@
       <c r="BC27" s="20"/>
       <c r="BD27" s="20"/>
       <c r="BE27" s="20"/>
-      <c r="BF27" s="20"/>
     </row>
     <row r="28" ht="12.75" customHeight="1">
       <c r="A28" s="20"/>
@@ -2475,7 +2441,6 @@
       <c r="BC28" s="20"/>
       <c r="BD28" s="20"/>
       <c r="BE28" s="20"/>
-      <c r="BF28" s="20"/>
     </row>
     <row r="29" ht="12.75" customHeight="1">
       <c r="A29" s="20"/>
@@ -2535,7 +2500,6 @@
       <c r="BC29" s="20"/>
       <c r="BD29" s="20"/>
       <c r="BE29" s="20"/>
-      <c r="BF29" s="20"/>
     </row>
     <row r="30" ht="12.75" customHeight="1">
       <c r="A30" s="20"/>
@@ -2595,7 +2559,6 @@
       <c r="BC30" s="20"/>
       <c r="BD30" s="20"/>
       <c r="BE30" s="20"/>
-      <c r="BF30" s="20"/>
     </row>
     <row r="31" ht="12.75" customHeight="1">
       <c r="A31" s="20"/>
@@ -2655,7 +2618,6 @@
       <c r="BC31" s="20"/>
       <c r="BD31" s="20"/>
       <c r="BE31" s="20"/>
-      <c r="BF31" s="20"/>
     </row>
     <row r="32" ht="12.75" customHeight="1">
       <c r="A32" s="20"/>
@@ -2715,7 +2677,6 @@
       <c r="BC32" s="20"/>
       <c r="BD32" s="20"/>
       <c r="BE32" s="20"/>
-      <c r="BF32" s="20"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="20"/>
@@ -2775,7 +2736,6 @@
       <c r="BC33" s="20"/>
       <c r="BD33" s="20"/>
       <c r="BE33" s="20"/>
-      <c r="BF33" s="20"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="20"/>
@@ -2835,7 +2795,6 @@
       <c r="BC34" s="20"/>
       <c r="BD34" s="20"/>
       <c r="BE34" s="20"/>
-      <c r="BF34" s="20"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="20"/>
@@ -2895,7 +2854,6 @@
       <c r="BC35" s="20"/>
       <c r="BD35" s="20"/>
       <c r="BE35" s="20"/>
-      <c r="BF35" s="20"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="20"/>
@@ -2955,7 +2913,6 @@
       <c r="BC36" s="20"/>
       <c r="BD36" s="20"/>
       <c r="BE36" s="20"/>
-      <c r="BF36" s="20"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="20"/>
@@ -3015,7 +2972,6 @@
       <c r="BC37" s="20"/>
       <c r="BD37" s="20"/>
       <c r="BE37" s="20"/>
-      <c r="BF37" s="20"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="20"/>
@@ -3075,7 +3031,6 @@
       <c r="BC38" s="20"/>
       <c r="BD38" s="20"/>
       <c r="BE38" s="20"/>
-      <c r="BF38" s="20"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
       <c r="A39" s="20"/>
@@ -3135,7 +3090,6 @@
       <c r="BC39" s="20"/>
       <c r="BD39" s="20"/>
       <c r="BE39" s="20"/>
-      <c r="BF39" s="20"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="20"/>
@@ -3195,7 +3149,6 @@
       <c r="BC40" s="20"/>
       <c r="BD40" s="20"/>
       <c r="BE40" s="20"/>
-      <c r="BF40" s="20"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="20"/>
@@ -3255,7 +3208,6 @@
       <c r="BC41" s="20"/>
       <c r="BD41" s="20"/>
       <c r="BE41" s="20"/>
-      <c r="BF41" s="20"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="20"/>
@@ -3315,7 +3267,6 @@
       <c r="BC42" s="20"/>
       <c r="BD42" s="20"/>
       <c r="BE42" s="20"/>
-      <c r="BF42" s="20"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="20"/>
@@ -3375,7 +3326,6 @@
       <c r="BC43" s="20"/>
       <c r="BD43" s="20"/>
       <c r="BE43" s="20"/>
-      <c r="BF43" s="20"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="20"/>
@@ -3435,7 +3385,6 @@
       <c r="BC44" s="20"/>
       <c r="BD44" s="20"/>
       <c r="BE44" s="20"/>
-      <c r="BF44" s="20"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="20"/>
@@ -3495,7 +3444,6 @@
       <c r="BC45" s="20"/>
       <c r="BD45" s="20"/>
       <c r="BE45" s="20"/>
-      <c r="BF45" s="20"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="20"/>
@@ -3555,7 +3503,6 @@
       <c r="BC46" s="20"/>
       <c r="BD46" s="20"/>
       <c r="BE46" s="20"/>
-      <c r="BF46" s="20"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="20"/>
@@ -3615,7 +3562,6 @@
       <c r="BC47" s="20"/>
       <c r="BD47" s="20"/>
       <c r="BE47" s="20"/>
-      <c r="BF47" s="20"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="20"/>
@@ -3675,7 +3621,6 @@
       <c r="BC48" s="20"/>
       <c r="BD48" s="20"/>
       <c r="BE48" s="20"/>
-      <c r="BF48" s="20"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="20"/>
@@ -3735,7 +3680,6 @@
       <c r="BC49" s="20"/>
       <c r="BD49" s="20"/>
       <c r="BE49" s="20"/>
-      <c r="BF49" s="20"/>
     </row>
     <row r="50" ht="12.75" customHeight="1">
       <c r="A50" s="20"/>
@@ -3795,7 +3739,6 @@
       <c r="BC50" s="20"/>
       <c r="BD50" s="20"/>
       <c r="BE50" s="20"/>
-      <c r="BF50" s="20"/>
     </row>
     <row r="51" ht="12.75" customHeight="1">
       <c r="A51" s="20"/>
@@ -3855,7 +3798,6 @@
       <c r="BC51" s="20"/>
       <c r="BD51" s="20"/>
       <c r="BE51" s="20"/>
-      <c r="BF51" s="20"/>
     </row>
     <row r="52" ht="12.75" customHeight="1">
       <c r="A52" s="20"/>
@@ -3915,7 +3857,6 @@
       <c r="BC52" s="20"/>
       <c r="BD52" s="20"/>
       <c r="BE52" s="20"/>
-      <c r="BF52" s="20"/>
     </row>
     <row r="53" ht="12.75" customHeight="1">
       <c r="A53" s="20"/>
@@ -3975,7 +3916,6 @@
       <c r="BC53" s="20"/>
       <c r="BD53" s="20"/>
       <c r="BE53" s="20"/>
-      <c r="BF53" s="20"/>
     </row>
     <row r="54" ht="12.75" customHeight="1">
       <c r="A54" s="20"/>
@@ -4035,7 +3975,6 @@
       <c r="BC54" s="20"/>
       <c r="BD54" s="20"/>
       <c r="BE54" s="20"/>
-      <c r="BF54" s="20"/>
     </row>
     <row r="55" ht="12.75" customHeight="1">
       <c r="A55" s="20"/>
@@ -4095,7 +4034,6 @@
       <c r="BC55" s="20"/>
       <c r="BD55" s="20"/>
       <c r="BE55" s="20"/>
-      <c r="BF55" s="20"/>
     </row>
     <row r="56" ht="12.75" customHeight="1">
       <c r="A56" s="20"/>
@@ -4155,7 +4093,6 @@
       <c r="BC56" s="20"/>
       <c r="BD56" s="20"/>
       <c r="BE56" s="20"/>
-      <c r="BF56" s="20"/>
     </row>
     <row r="57" ht="12.75" customHeight="1">
       <c r="A57" s="20"/>
@@ -4215,7 +4152,6 @@
       <c r="BC57" s="20"/>
       <c r="BD57" s="20"/>
       <c r="BE57" s="20"/>
-      <c r="BF57" s="20"/>
     </row>
     <row r="58" ht="12.75" customHeight="1">
       <c r="A58" s="20"/>
@@ -4275,7 +4211,6 @@
       <c r="BC58" s="20"/>
       <c r="BD58" s="20"/>
       <c r="BE58" s="20"/>
-      <c r="BF58" s="20"/>
     </row>
     <row r="59" ht="12.75" customHeight="1">
       <c r="A59" s="20"/>
@@ -4335,7 +4270,6 @@
       <c r="BC59" s="20"/>
       <c r="BD59" s="20"/>
       <c r="BE59" s="20"/>
-      <c r="BF59" s="20"/>
     </row>
     <row r="60" ht="12.75" customHeight="1">
       <c r="A60" s="20"/>
@@ -4395,7 +4329,6 @@
       <c r="BC60" s="20"/>
       <c r="BD60" s="20"/>
       <c r="BE60" s="20"/>
-      <c r="BF60" s="20"/>
     </row>
     <row r="61" ht="12.75" customHeight="1">
       <c r="A61" s="20"/>
@@ -4455,7 +4388,6 @@
       <c r="BC61" s="20"/>
       <c r="BD61" s="20"/>
       <c r="BE61" s="20"/>
-      <c r="BF61" s="20"/>
     </row>
     <row r="62" ht="12.75" customHeight="1">
       <c r="A62" s="20"/>
@@ -4515,7 +4447,6 @@
       <c r="BC62" s="20"/>
       <c r="BD62" s="20"/>
       <c r="BE62" s="20"/>
-      <c r="BF62" s="20"/>
     </row>
     <row r="63" ht="12.75" customHeight="1">
       <c r="A63" s="20"/>
@@ -4575,7 +4506,6 @@
       <c r="BC63" s="20"/>
       <c r="BD63" s="20"/>
       <c r="BE63" s="20"/>
-      <c r="BF63" s="20"/>
     </row>
     <row r="64" ht="12.75" customHeight="1">
       <c r="A64" s="20"/>
@@ -4635,7 +4565,6 @@
       <c r="BC64" s="20"/>
       <c r="BD64" s="20"/>
       <c r="BE64" s="20"/>
-      <c r="BF64" s="20"/>
     </row>
     <row r="65" ht="12.75" customHeight="1">
       <c r="A65" s="20"/>
@@ -4695,7 +4624,6 @@
       <c r="BC65" s="20"/>
       <c r="BD65" s="20"/>
       <c r="BE65" s="20"/>
-      <c r="BF65" s="20"/>
     </row>
     <row r="66" ht="12.75" customHeight="1">
       <c r="A66" s="20"/>
@@ -4755,7 +4683,6 @@
       <c r="BC66" s="20"/>
       <c r="BD66" s="20"/>
       <c r="BE66" s="20"/>
-      <c r="BF66" s="20"/>
     </row>
     <row r="67" ht="12.75" customHeight="1">
       <c r="A67" s="20"/>
@@ -4815,7 +4742,6 @@
       <c r="BC67" s="20"/>
       <c r="BD67" s="20"/>
       <c r="BE67" s="20"/>
-      <c r="BF67" s="20"/>
     </row>
     <row r="68" ht="12.75" customHeight="1">
       <c r="A68" s="20"/>
@@ -4875,7 +4801,6 @@
       <c r="BC68" s="20"/>
       <c r="BD68" s="20"/>
       <c r="BE68" s="20"/>
-      <c r="BF68" s="20"/>
     </row>
     <row r="69" ht="12.75" customHeight="1">
       <c r="A69" s="20"/>
@@ -4935,7 +4860,6 @@
       <c r="BC69" s="20"/>
       <c r="BD69" s="20"/>
       <c r="BE69" s="20"/>
-      <c r="BF69" s="20"/>
     </row>
     <row r="70" ht="12.75" customHeight="1">
       <c r="A70" s="20"/>
@@ -4995,7 +4919,6 @@
       <c r="BC70" s="20"/>
       <c r="BD70" s="20"/>
       <c r="BE70" s="20"/>
-      <c r="BF70" s="20"/>
     </row>
     <row r="71" ht="12.75" customHeight="1">
       <c r="A71" s="20"/>
@@ -5055,7 +4978,6 @@
       <c r="BC71" s="20"/>
       <c r="BD71" s="20"/>
       <c r="BE71" s="20"/>
-      <c r="BF71" s="20"/>
     </row>
     <row r="72" ht="12.75" customHeight="1">
       <c r="A72" s="20"/>
@@ -5115,7 +5037,6 @@
       <c r="BC72" s="20"/>
       <c r="BD72" s="20"/>
       <c r="BE72" s="20"/>
-      <c r="BF72" s="20"/>
     </row>
     <row r="73" ht="12.75" customHeight="1">
       <c r="A73" s="20"/>
@@ -5175,7 +5096,6 @@
       <c r="BC73" s="20"/>
       <c r="BD73" s="20"/>
       <c r="BE73" s="20"/>
-      <c r="BF73" s="20"/>
     </row>
     <row r="74" ht="12.75" customHeight="1">
       <c r="A74" s="20"/>
@@ -5235,7 +5155,6 @@
       <c r="BC74" s="20"/>
       <c r="BD74" s="20"/>
       <c r="BE74" s="20"/>
-      <c r="BF74" s="20"/>
     </row>
     <row r="75" ht="12.75" customHeight="1">
       <c r="A75" s="20"/>
@@ -5295,7 +5214,6 @@
       <c r="BC75" s="20"/>
       <c r="BD75" s="20"/>
       <c r="BE75" s="20"/>
-      <c r="BF75" s="20"/>
     </row>
     <row r="76" ht="12.75" customHeight="1">
       <c r="A76" s="20"/>
@@ -5355,7 +5273,6 @@
       <c r="BC76" s="20"/>
       <c r="BD76" s="20"/>
       <c r="BE76" s="20"/>
-      <c r="BF76" s="20"/>
     </row>
     <row r="77" ht="12.75" customHeight="1">
       <c r="A77" s="20"/>
@@ -5415,7 +5332,6 @@
       <c r="BC77" s="20"/>
       <c r="BD77" s="20"/>
       <c r="BE77" s="20"/>
-      <c r="BF77" s="20"/>
     </row>
     <row r="78" ht="12.75" customHeight="1">
       <c r="A78" s="20"/>
@@ -5475,7 +5391,6 @@
       <c r="BC78" s="20"/>
       <c r="BD78" s="20"/>
       <c r="BE78" s="20"/>
-      <c r="BF78" s="20"/>
     </row>
     <row r="79" ht="12.75" customHeight="1">
       <c r="A79" s="20"/>
@@ -5535,7 +5450,6 @@
       <c r="BC79" s="20"/>
       <c r="BD79" s="20"/>
       <c r="BE79" s="20"/>
-      <c r="BF79" s="20"/>
     </row>
     <row r="80" ht="12.75" customHeight="1">
       <c r="A80" s="20"/>
@@ -5595,7 +5509,6 @@
       <c r="BC80" s="20"/>
       <c r="BD80" s="20"/>
       <c r="BE80" s="20"/>
-      <c r="BF80" s="20"/>
     </row>
     <row r="81" ht="12.75" customHeight="1">
       <c r="A81" s="20"/>
@@ -5655,7 +5568,6 @@
       <c r="BC81" s="20"/>
       <c r="BD81" s="20"/>
       <c r="BE81" s="20"/>
-      <c r="BF81" s="20"/>
     </row>
     <row r="82" ht="12.75" customHeight="1">
       <c r="A82" s="20"/>
@@ -5715,7 +5627,6 @@
       <c r="BC82" s="20"/>
       <c r="BD82" s="20"/>
       <c r="BE82" s="20"/>
-      <c r="BF82" s="20"/>
     </row>
     <row r="83" ht="12.75" customHeight="1">
       <c r="A83" s="20"/>
@@ -5775,7 +5686,6 @@
       <c r="BC83" s="20"/>
       <c r="BD83" s="20"/>
       <c r="BE83" s="20"/>
-      <c r="BF83" s="20"/>
     </row>
     <row r="84" ht="12.75" customHeight="1">
       <c r="A84" s="20"/>
@@ -5835,7 +5745,6 @@
       <c r="BC84" s="20"/>
       <c r="BD84" s="20"/>
       <c r="BE84" s="20"/>
-      <c r="BF84" s="20"/>
     </row>
     <row r="85" ht="12.75" customHeight="1">
       <c r="A85" s="20"/>
@@ -5895,7 +5804,6 @@
       <c r="BC85" s="20"/>
       <c r="BD85" s="20"/>
       <c r="BE85" s="20"/>
-      <c r="BF85" s="20"/>
     </row>
     <row r="86" ht="12.75" customHeight="1">
       <c r="A86" s="20"/>
@@ -5955,7 +5863,6 @@
       <c r="BC86" s="20"/>
       <c r="BD86" s="20"/>
       <c r="BE86" s="20"/>
-      <c r="BF86" s="20"/>
     </row>
     <row r="87" ht="12.75" customHeight="1">
       <c r="A87" s="20"/>
@@ -6015,7 +5922,6 @@
       <c r="BC87" s="20"/>
       <c r="BD87" s="20"/>
       <c r="BE87" s="20"/>
-      <c r="BF87" s="20"/>
     </row>
     <row r="88" ht="12.75" customHeight="1">
       <c r="A88" s="20"/>
@@ -6075,7 +5981,6 @@
       <c r="BC88" s="20"/>
       <c r="BD88" s="20"/>
       <c r="BE88" s="20"/>
-      <c r="BF88" s="20"/>
     </row>
     <row r="89" ht="12.75" customHeight="1">
       <c r="A89" s="20"/>
@@ -6135,7 +6040,6 @@
       <c r="BC89" s="20"/>
       <c r="BD89" s="20"/>
       <c r="BE89" s="20"/>
-      <c r="BF89" s="20"/>
     </row>
     <row r="90" ht="12.75" customHeight="1">
       <c r="A90" s="20"/>
@@ -6195,7 +6099,6 @@
       <c r="BC90" s="20"/>
       <c r="BD90" s="20"/>
       <c r="BE90" s="20"/>
-      <c r="BF90" s="20"/>
     </row>
     <row r="91" ht="12.75" customHeight="1">
       <c r="A91" s="20"/>
@@ -6255,7 +6158,6 @@
       <c r="BC91" s="20"/>
       <c r="BD91" s="20"/>
       <c r="BE91" s="20"/>
-      <c r="BF91" s="20"/>
     </row>
     <row r="92" ht="12.75" customHeight="1">
       <c r="A92" s="20"/>
@@ -6315,7 +6217,6 @@
       <c r="BC92" s="20"/>
       <c r="BD92" s="20"/>
       <c r="BE92" s="20"/>
-      <c r="BF92" s="20"/>
     </row>
     <row r="93" ht="12.75" customHeight="1">
       <c r="A93" s="20"/>
@@ -6375,7 +6276,6 @@
       <c r="BC93" s="20"/>
       <c r="BD93" s="20"/>
       <c r="BE93" s="20"/>
-      <c r="BF93" s="20"/>
     </row>
     <row r="94" ht="12.75" customHeight="1">
       <c r="A94" s="20"/>
@@ -6435,7 +6335,6 @@
       <c r="BC94" s="20"/>
       <c r="BD94" s="20"/>
       <c r="BE94" s="20"/>
-      <c r="BF94" s="20"/>
     </row>
     <row r="95" ht="12.75" customHeight="1">
       <c r="A95" s="20"/>
@@ -6495,7 +6394,6 @@
       <c r="BC95" s="20"/>
       <c r="BD95" s="20"/>
       <c r="BE95" s="20"/>
-      <c r="BF95" s="20"/>
     </row>
     <row r="96" ht="12.75" customHeight="1">
       <c r="A96" s="20"/>
@@ -6555,7 +6453,6 @@
       <c r="BC96" s="20"/>
       <c r="BD96" s="20"/>
       <c r="BE96" s="20"/>
-      <c r="BF96" s="20"/>
     </row>
     <row r="97" ht="12.75" customHeight="1">
       <c r="A97" s="20"/>
@@ -6615,7 +6512,6 @@
       <c r="BC97" s="20"/>
       <c r="BD97" s="20"/>
       <c r="BE97" s="20"/>
-      <c r="BF97" s="20"/>
     </row>
     <row r="98" ht="12.75" customHeight="1">
       <c r="A98" s="20"/>
@@ -6675,7 +6571,6 @@
       <c r="BC98" s="20"/>
       <c r="BD98" s="20"/>
       <c r="BE98" s="20"/>
-      <c r="BF98" s="20"/>
     </row>
     <row r="99" ht="12.75" customHeight="1">
       <c r="A99" s="20"/>
@@ -6735,7 +6630,6 @@
       <c r="BC99" s="20"/>
       <c r="BD99" s="20"/>
       <c r="BE99" s="20"/>
-      <c r="BF99" s="20"/>
     </row>
     <row r="100" ht="12.75" customHeight="1">
       <c r="A100" s="20"/>
@@ -6795,7 +6689,6 @@
       <c r="BC100" s="20"/>
       <c r="BD100" s="20"/>
       <c r="BE100" s="20"/>
-      <c r="BF100" s="20"/>
     </row>
     <row r="101" ht="12.75" customHeight="1">
       <c r="A101" s="20"/>
@@ -6855,7 +6748,6 @@
       <c r="BC101" s="20"/>
       <c r="BD101" s="20"/>
       <c r="BE101" s="20"/>
-      <c r="BF101" s="20"/>
     </row>
     <row r="102" ht="12.75" customHeight="1">
       <c r="A102" s="20"/>
@@ -6915,7 +6807,6 @@
       <c r="BC102" s="20"/>
       <c r="BD102" s="20"/>
       <c r="BE102" s="20"/>
-      <c r="BF102" s="20"/>
     </row>
     <row r="103" ht="12.75" customHeight="1">
       <c r="A103" s="20"/>
@@ -6975,7 +6866,6 @@
       <c r="BC103" s="20"/>
       <c r="BD103" s="20"/>
       <c r="BE103" s="20"/>
-      <c r="BF103" s="20"/>
     </row>
     <row r="104" ht="12.75" customHeight="1">
       <c r="A104" s="20"/>
@@ -7035,7 +6925,6 @@
       <c r="BC104" s="20"/>
       <c r="BD104" s="20"/>
       <c r="BE104" s="20"/>
-      <c r="BF104" s="20"/>
     </row>
     <row r="105" ht="12.75" customHeight="1">
       <c r="A105" s="20"/>
@@ -7095,7 +6984,6 @@
       <c r="BC105" s="20"/>
       <c r="BD105" s="20"/>
       <c r="BE105" s="20"/>
-      <c r="BF105" s="20"/>
     </row>
     <row r="106" ht="12.75" customHeight="1">
       <c r="A106" s="20"/>
@@ -7155,7 +7043,6 @@
       <c r="BC106" s="20"/>
       <c r="BD106" s="20"/>
       <c r="BE106" s="20"/>
-      <c r="BF106" s="20"/>
     </row>
     <row r="107" ht="12.75" customHeight="1">
       <c r="A107" s="20"/>
@@ -7215,7 +7102,6 @@
       <c r="BC107" s="20"/>
       <c r="BD107" s="20"/>
       <c r="BE107" s="20"/>
-      <c r="BF107" s="20"/>
     </row>
     <row r="108" ht="12.75" customHeight="1">
       <c r="A108" s="20"/>
@@ -7275,7 +7161,6 @@
       <c r="BC108" s="20"/>
       <c r="BD108" s="20"/>
       <c r="BE108" s="20"/>
-      <c r="BF108" s="20"/>
     </row>
     <row r="109" ht="12.75" customHeight="1">
       <c r="A109" s="20"/>
@@ -7335,7 +7220,6 @@
       <c r="BC109" s="20"/>
       <c r="BD109" s="20"/>
       <c r="BE109" s="20"/>
-      <c r="BF109" s="20"/>
     </row>
     <row r="110" ht="12.75" customHeight="1">
       <c r="A110" s="20"/>
@@ -7395,7 +7279,6 @@
       <c r="BC110" s="20"/>
       <c r="BD110" s="20"/>
       <c r="BE110" s="20"/>
-      <c r="BF110" s="20"/>
     </row>
     <row r="111" ht="12.75" customHeight="1">
       <c r="A111" s="20"/>
@@ -7455,7 +7338,6 @@
       <c r="BC111" s="20"/>
       <c r="BD111" s="20"/>
       <c r="BE111" s="20"/>
-      <c r="BF111" s="20"/>
     </row>
     <row r="112" ht="12.75" customHeight="1">
       <c r="A112" s="20"/>
@@ -7515,7 +7397,6 @@
       <c r="BC112" s="20"/>
       <c r="BD112" s="20"/>
       <c r="BE112" s="20"/>
-      <c r="BF112" s="20"/>
     </row>
     <row r="113" ht="12.75" customHeight="1">
       <c r="A113" s="20"/>
@@ -7575,7 +7456,6 @@
       <c r="BC113" s="20"/>
       <c r="BD113" s="20"/>
       <c r="BE113" s="20"/>
-      <c r="BF113" s="20"/>
     </row>
     <row r="114" ht="12.75" customHeight="1">
       <c r="A114" s="20"/>
@@ -7635,7 +7515,6 @@
       <c r="BC114" s="20"/>
       <c r="BD114" s="20"/>
       <c r="BE114" s="20"/>
-      <c r="BF114" s="20"/>
     </row>
     <row r="115" ht="12.75" customHeight="1">
       <c r="A115" s="20"/>
@@ -7695,7 +7574,6 @@
       <c r="BC115" s="20"/>
       <c r="BD115" s="20"/>
       <c r="BE115" s="20"/>
-      <c r="BF115" s="20"/>
     </row>
     <row r="116" ht="12.75" customHeight="1">
       <c r="A116" s="20"/>
@@ -7755,7 +7633,6 @@
       <c r="BC116" s="20"/>
       <c r="BD116" s="20"/>
       <c r="BE116" s="20"/>
-      <c r="BF116" s="20"/>
     </row>
     <row r="117" ht="12.75" customHeight="1">
       <c r="A117" s="20"/>
@@ -7815,7 +7692,6 @@
       <c r="BC117" s="20"/>
       <c r="BD117" s="20"/>
       <c r="BE117" s="20"/>
-      <c r="BF117" s="20"/>
     </row>
     <row r="118" ht="12.75" customHeight="1">
       <c r="A118" s="20"/>
@@ -7875,7 +7751,6 @@
       <c r="BC118" s="20"/>
       <c r="BD118" s="20"/>
       <c r="BE118" s="20"/>
-      <c r="BF118" s="20"/>
     </row>
     <row r="119" ht="12.75" customHeight="1">
       <c r="A119" s="20"/>
@@ -7935,7 +7810,6 @@
       <c r="BC119" s="20"/>
       <c r="BD119" s="20"/>
       <c r="BE119" s="20"/>
-      <c r="BF119" s="20"/>
     </row>
     <row r="120" ht="12.75" customHeight="1">
       <c r="A120" s="20"/>
@@ -7995,7 +7869,6 @@
       <c r="BC120" s="20"/>
       <c r="BD120" s="20"/>
       <c r="BE120" s="20"/>
-      <c r="BF120" s="20"/>
     </row>
     <row r="121" ht="12.75" customHeight="1">
       <c r="A121" s="20"/>
@@ -8055,7 +7928,6 @@
       <c r="BC121" s="20"/>
       <c r="BD121" s="20"/>
       <c r="BE121" s="20"/>
-      <c r="BF121" s="20"/>
     </row>
     <row r="122" ht="12.75" customHeight="1">
       <c r="A122" s="20"/>
@@ -8115,7 +7987,6 @@
       <c r="BC122" s="20"/>
       <c r="BD122" s="20"/>
       <c r="BE122" s="20"/>
-      <c r="BF122" s="20"/>
     </row>
     <row r="123" ht="12.75" customHeight="1">
       <c r="A123" s="20"/>
@@ -8175,7 +8046,6 @@
       <c r="BC123" s="20"/>
       <c r="BD123" s="20"/>
       <c r="BE123" s="20"/>
-      <c r="BF123" s="20"/>
     </row>
     <row r="124" ht="12.75" customHeight="1">
       <c r="A124" s="20"/>
@@ -8235,7 +8105,6 @@
       <c r="BC124" s="20"/>
       <c r="BD124" s="20"/>
       <c r="BE124" s="20"/>
-      <c r="BF124" s="20"/>
     </row>
     <row r="125" ht="12.75" customHeight="1">
       <c r="A125" s="20"/>
@@ -8295,7 +8164,6 @@
       <c r="BC125" s="20"/>
       <c r="BD125" s="20"/>
       <c r="BE125" s="20"/>
-      <c r="BF125" s="20"/>
     </row>
     <row r="126" ht="12.75" customHeight="1">
       <c r="A126" s="20"/>
@@ -8355,7 +8223,6 @@
       <c r="BC126" s="20"/>
       <c r="BD126" s="20"/>
       <c r="BE126" s="20"/>
-      <c r="BF126" s="20"/>
     </row>
     <row r="127" ht="12.75" customHeight="1">
       <c r="A127" s="20"/>
@@ -8415,7 +8282,6 @@
       <c r="BC127" s="20"/>
       <c r="BD127" s="20"/>
       <c r="BE127" s="20"/>
-      <c r="BF127" s="20"/>
     </row>
     <row r="128" ht="12.75" customHeight="1">
       <c r="A128" s="20"/>
@@ -8475,7 +8341,6 @@
       <c r="BC128" s="20"/>
       <c r="BD128" s="20"/>
       <c r="BE128" s="20"/>
-      <c r="BF128" s="20"/>
     </row>
     <row r="129" ht="12.75" customHeight="1">
       <c r="A129" s="20"/>
@@ -8535,7 +8400,6 @@
       <c r="BC129" s="20"/>
       <c r="BD129" s="20"/>
       <c r="BE129" s="20"/>
-      <c r="BF129" s="20"/>
     </row>
     <row r="130" ht="12.75" customHeight="1">
       <c r="A130" s="20"/>
@@ -8595,7 +8459,6 @@
       <c r="BC130" s="20"/>
       <c r="BD130" s="20"/>
       <c r="BE130" s="20"/>
-      <c r="BF130" s="20"/>
     </row>
     <row r="131" ht="12.75" customHeight="1">
       <c r="A131" s="20"/>
@@ -8655,7 +8518,6 @@
       <c r="BC131" s="20"/>
       <c r="BD131" s="20"/>
       <c r="BE131" s="20"/>
-      <c r="BF131" s="20"/>
     </row>
     <row r="132" ht="12.75" customHeight="1">
       <c r="A132" s="20"/>
@@ -8715,7 +8577,6 @@
       <c r="BC132" s="20"/>
       <c r="BD132" s="20"/>
       <c r="BE132" s="20"/>
-      <c r="BF132" s="20"/>
     </row>
     <row r="133" ht="12.75" customHeight="1">
       <c r="A133" s="20"/>
@@ -8775,7 +8636,6 @@
       <c r="BC133" s="20"/>
       <c r="BD133" s="20"/>
       <c r="BE133" s="20"/>
-      <c r="BF133" s="20"/>
     </row>
     <row r="134" ht="12.75" customHeight="1">
       <c r="A134" s="20"/>
@@ -8835,7 +8695,6 @@
       <c r="BC134" s="20"/>
       <c r="BD134" s="20"/>
       <c r="BE134" s="20"/>
-      <c r="BF134" s="20"/>
     </row>
     <row r="135" ht="12.75" customHeight="1">
       <c r="A135" s="20"/>
@@ -8895,7 +8754,6 @@
       <c r="BC135" s="20"/>
       <c r="BD135" s="20"/>
       <c r="BE135" s="20"/>
-      <c r="BF135" s="20"/>
     </row>
     <row r="136" ht="12.75" customHeight="1">
       <c r="A136" s="20"/>
@@ -8955,7 +8813,6 @@
       <c r="BC136" s="20"/>
       <c r="BD136" s="20"/>
       <c r="BE136" s="20"/>
-      <c r="BF136" s="20"/>
     </row>
     <row r="137" ht="12.75" customHeight="1">
       <c r="A137" s="20"/>
@@ -9015,7 +8872,6 @@
       <c r="BC137" s="20"/>
       <c r="BD137" s="20"/>
       <c r="BE137" s="20"/>
-      <c r="BF137" s="20"/>
     </row>
     <row r="138" ht="12.75" customHeight="1">
       <c r="A138" s="20"/>
@@ -9075,7 +8931,6 @@
       <c r="BC138" s="20"/>
       <c r="BD138" s="20"/>
       <c r="BE138" s="20"/>
-      <c r="BF138" s="20"/>
     </row>
     <row r="139" ht="12.75" customHeight="1">
       <c r="A139" s="20"/>
@@ -9135,7 +8990,6 @@
       <c r="BC139" s="20"/>
       <c r="BD139" s="20"/>
       <c r="BE139" s="20"/>
-      <c r="BF139" s="20"/>
     </row>
     <row r="140" ht="12.75" customHeight="1">
       <c r="A140" s="20"/>
@@ -9195,7 +9049,6 @@
       <c r="BC140" s="20"/>
       <c r="BD140" s="20"/>
       <c r="BE140" s="20"/>
-      <c r="BF140" s="20"/>
     </row>
     <row r="141" ht="12.75" customHeight="1">
       <c r="A141" s="20"/>
@@ -9255,7 +9108,6 @@
       <c r="BC141" s="20"/>
       <c r="BD141" s="20"/>
       <c r="BE141" s="20"/>
-      <c r="BF141" s="20"/>
     </row>
     <row r="142" ht="12.75" customHeight="1">
       <c r="A142" s="20"/>
@@ -9315,7 +9167,6 @@
       <c r="BC142" s="20"/>
       <c r="BD142" s="20"/>
       <c r="BE142" s="20"/>
-      <c r="BF142" s="20"/>
     </row>
     <row r="143" ht="12.75" customHeight="1">
       <c r="A143" s="20"/>
@@ -9375,7 +9226,6 @@
       <c r="BC143" s="20"/>
       <c r="BD143" s="20"/>
       <c r="BE143" s="20"/>
-      <c r="BF143" s="20"/>
     </row>
     <row r="144" ht="12.75" customHeight="1">
       <c r="A144" s="20"/>
@@ -9435,7 +9285,6 @@
       <c r="BC144" s="20"/>
       <c r="BD144" s="20"/>
       <c r="BE144" s="20"/>
-      <c r="BF144" s="20"/>
     </row>
     <row r="145" ht="12.75" customHeight="1">
       <c r="A145" s="20"/>
@@ -9495,7 +9344,6 @@
       <c r="BC145" s="20"/>
       <c r="BD145" s="20"/>
       <c r="BE145" s="20"/>
-      <c r="BF145" s="20"/>
     </row>
     <row r="146" ht="12.75" customHeight="1">
       <c r="A146" s="20"/>
@@ -9555,7 +9403,6 @@
       <c r="BC146" s="20"/>
       <c r="BD146" s="20"/>
       <c r="BE146" s="20"/>
-      <c r="BF146" s="20"/>
     </row>
     <row r="147" ht="12.75" customHeight="1">
       <c r="A147" s="20"/>
@@ -9615,7 +9462,6 @@
       <c r="BC147" s="20"/>
       <c r="BD147" s="20"/>
       <c r="BE147" s="20"/>
-      <c r="BF147" s="20"/>
     </row>
     <row r="148" ht="12.75" customHeight="1">
       <c r="A148" s="20"/>
@@ -9675,7 +9521,6 @@
       <c r="BC148" s="20"/>
       <c r="BD148" s="20"/>
       <c r="BE148" s="20"/>
-      <c r="BF148" s="20"/>
     </row>
     <row r="149" ht="12.75" customHeight="1">
       <c r="A149" s="20"/>
@@ -9735,7 +9580,6 @@
       <c r="BC149" s="20"/>
       <c r="BD149" s="20"/>
       <c r="BE149" s="20"/>
-      <c r="BF149" s="20"/>
     </row>
     <row r="150" ht="12.75" customHeight="1">
       <c r="A150" s="20"/>
@@ -9795,7 +9639,6 @@
       <c r="BC150" s="20"/>
       <c r="BD150" s="20"/>
       <c r="BE150" s="20"/>
-      <c r="BF150" s="20"/>
     </row>
     <row r="151" ht="12.75" customHeight="1">
       <c r="A151" s="20"/>
@@ -9855,7 +9698,6 @@
       <c r="BC151" s="20"/>
       <c r="BD151" s="20"/>
       <c r="BE151" s="20"/>
-      <c r="BF151" s="20"/>
     </row>
     <row r="152" ht="12.75" customHeight="1">
       <c r="A152" s="20"/>
@@ -9915,7 +9757,6 @@
       <c r="BC152" s="20"/>
       <c r="BD152" s="20"/>
       <c r="BE152" s="20"/>
-      <c r="BF152" s="20"/>
     </row>
     <row r="153" ht="12.75" customHeight="1">
       <c r="A153" s="20"/>
@@ -9975,7 +9816,6 @@
       <c r="BC153" s="20"/>
       <c r="BD153" s="20"/>
       <c r="BE153" s="20"/>
-      <c r="BF153" s="20"/>
     </row>
     <row r="154" ht="12.75" customHeight="1">
       <c r="A154" s="20"/>
@@ -10035,7 +9875,6 @@
       <c r="BC154" s="20"/>
       <c r="BD154" s="20"/>
       <c r="BE154" s="20"/>
-      <c r="BF154" s="20"/>
     </row>
     <row r="155" ht="12.75" customHeight="1">
       <c r="A155" s="20"/>
@@ -10095,7 +9934,6 @@
       <c r="BC155" s="20"/>
       <c r="BD155" s="20"/>
       <c r="BE155" s="20"/>
-      <c r="BF155" s="20"/>
     </row>
     <row r="156" ht="12.75" customHeight="1">
       <c r="A156" s="20"/>
@@ -10155,7 +9993,6 @@
       <c r="BC156" s="20"/>
       <c r="BD156" s="20"/>
       <c r="BE156" s="20"/>
-      <c r="BF156" s="20"/>
     </row>
     <row r="157" ht="12.75" customHeight="1">
       <c r="A157" s="20"/>
@@ -10215,7 +10052,6 @@
       <c r="BC157" s="20"/>
       <c r="BD157" s="20"/>
       <c r="BE157" s="20"/>
-      <c r="BF157" s="20"/>
     </row>
     <row r="158" ht="12.75" customHeight="1">
       <c r="A158" s="20"/>
@@ -10275,7 +10111,6 @@
       <c r="BC158" s="20"/>
       <c r="BD158" s="20"/>
       <c r="BE158" s="20"/>
-      <c r="BF158" s="20"/>
     </row>
     <row r="159" ht="12.75" customHeight="1">
       <c r="A159" s="20"/>
@@ -10335,7 +10170,6 @@
       <c r="BC159" s="20"/>
       <c r="BD159" s="20"/>
       <c r="BE159" s="20"/>
-      <c r="BF159" s="20"/>
     </row>
     <row r="160" ht="12.75" customHeight="1">
       <c r="A160" s="20"/>
@@ -10395,7 +10229,6 @@
       <c r="BC160" s="20"/>
       <c r="BD160" s="20"/>
       <c r="BE160" s="20"/>
-      <c r="BF160" s="20"/>
     </row>
     <row r="161" ht="12.75" customHeight="1">
       <c r="A161" s="20"/>
@@ -10455,7 +10288,6 @@
       <c r="BC161" s="20"/>
       <c r="BD161" s="20"/>
       <c r="BE161" s="20"/>
-      <c r="BF161" s="20"/>
     </row>
     <row r="162" ht="12.75" customHeight="1">
       <c r="A162" s="20"/>
@@ -10515,7 +10347,6 @@
       <c r="BC162" s="20"/>
       <c r="BD162" s="20"/>
       <c r="BE162" s="20"/>
-      <c r="BF162" s="20"/>
     </row>
     <row r="163" ht="12.75" customHeight="1">
       <c r="A163" s="20"/>
@@ -10575,7 +10406,6 @@
       <c r="BC163" s="20"/>
       <c r="BD163" s="20"/>
       <c r="BE163" s="20"/>
-      <c r="BF163" s="20"/>
     </row>
     <row r="164" ht="12.75" customHeight="1">
       <c r="A164" s="20"/>
@@ -10635,7 +10465,6 @@
       <c r="BC164" s="20"/>
       <c r="BD164" s="20"/>
       <c r="BE164" s="20"/>
-      <c r="BF164" s="20"/>
     </row>
     <row r="165" ht="12.75" customHeight="1">
       <c r="A165" s="20"/>
@@ -10695,7 +10524,6 @@
       <c r="BC165" s="20"/>
       <c r="BD165" s="20"/>
       <c r="BE165" s="20"/>
-      <c r="BF165" s="20"/>
     </row>
     <row r="166" ht="12.75" customHeight="1">
       <c r="A166" s="20"/>
@@ -10755,7 +10583,6 @@
       <c r="BC166" s="20"/>
       <c r="BD166" s="20"/>
       <c r="BE166" s="20"/>
-      <c r="BF166" s="20"/>
     </row>
     <row r="167" ht="12.75" customHeight="1">
       <c r="A167" s="20"/>
@@ -10815,7 +10642,6 @@
       <c r="BC167" s="20"/>
       <c r="BD167" s="20"/>
       <c r="BE167" s="20"/>
-      <c r="BF167" s="20"/>
     </row>
     <row r="168" ht="12.75" customHeight="1">
       <c r="A168" s="20"/>
@@ -10875,7 +10701,6 @@
       <c r="BC168" s="20"/>
       <c r="BD168" s="20"/>
       <c r="BE168" s="20"/>
-      <c r="BF168" s="20"/>
     </row>
     <row r="169" ht="12.75" customHeight="1">
       <c r="A169" s="20"/>
@@ -10935,7 +10760,6 @@
       <c r="BC169" s="20"/>
       <c r="BD169" s="20"/>
       <c r="BE169" s="20"/>
-      <c r="BF169" s="20"/>
     </row>
     <row r="170" ht="12.75" customHeight="1">
       <c r="A170" s="20"/>
@@ -10995,7 +10819,6 @@
       <c r="BC170" s="20"/>
       <c r="BD170" s="20"/>
       <c r="BE170" s="20"/>
-      <c r="BF170" s="20"/>
     </row>
     <row r="171" ht="12.75" customHeight="1">
       <c r="A171" s="20"/>
@@ -11055,7 +10878,6 @@
       <c r="BC171" s="20"/>
       <c r="BD171" s="20"/>
       <c r="BE171" s="20"/>
-      <c r="BF171" s="20"/>
     </row>
     <row r="172" ht="12.75" customHeight="1">
       <c r="A172" s="20"/>
@@ -11115,7 +10937,6 @@
       <c r="BC172" s="20"/>
       <c r="BD172" s="20"/>
       <c r="BE172" s="20"/>
-      <c r="BF172" s="20"/>
     </row>
     <row r="173" ht="12.75" customHeight="1">
       <c r="A173" s="20"/>
@@ -11175,7 +10996,6 @@
       <c r="BC173" s="20"/>
       <c r="BD173" s="20"/>
       <c r="BE173" s="20"/>
-      <c r="BF173" s="20"/>
     </row>
     <row r="174" ht="12.75" customHeight="1">
       <c r="A174" s="20"/>
@@ -11235,7 +11055,6 @@
       <c r="BC174" s="20"/>
       <c r="BD174" s="20"/>
       <c r="BE174" s="20"/>
-      <c r="BF174" s="20"/>
     </row>
     <row r="175" ht="12.75" customHeight="1">
       <c r="A175" s="20"/>
@@ -11295,7 +11114,6 @@
       <c r="BC175" s="20"/>
       <c r="BD175" s="20"/>
       <c r="BE175" s="20"/>
-      <c r="BF175" s="20"/>
     </row>
     <row r="176" ht="12.75" customHeight="1">
       <c r="A176" s="20"/>
@@ -11355,7 +11173,6 @@
       <c r="BC176" s="20"/>
       <c r="BD176" s="20"/>
       <c r="BE176" s="20"/>
-      <c r="BF176" s="20"/>
     </row>
     <row r="177" ht="12.75" customHeight="1">
       <c r="A177" s="20"/>
@@ -11415,7 +11232,6 @@
       <c r="BC177" s="20"/>
       <c r="BD177" s="20"/>
       <c r="BE177" s="20"/>
-      <c r="BF177" s="20"/>
     </row>
     <row r="178" ht="12.75" customHeight="1">
       <c r="A178" s="20"/>
@@ -11475,7 +11291,6 @@
       <c r="BC178" s="20"/>
       <c r="BD178" s="20"/>
       <c r="BE178" s="20"/>
-      <c r="BF178" s="20"/>
     </row>
     <row r="179" ht="12.75" customHeight="1">
       <c r="A179" s="20"/>
@@ -11535,7 +11350,6 @@
       <c r="BC179" s="20"/>
       <c r="BD179" s="20"/>
       <c r="BE179" s="20"/>
-      <c r="BF179" s="20"/>
     </row>
     <row r="180" ht="12.75" customHeight="1">
       <c r="A180" s="20"/>
@@ -11595,7 +11409,6 @@
       <c r="BC180" s="20"/>
       <c r="BD180" s="20"/>
       <c r="BE180" s="20"/>
-      <c r="BF180" s="20"/>
     </row>
     <row r="181" ht="12.75" customHeight="1">
       <c r="A181" s="20"/>
@@ -11655,7 +11468,6 @@
       <c r="BC181" s="20"/>
       <c r="BD181" s="20"/>
       <c r="BE181" s="20"/>
-      <c r="BF181" s="20"/>
     </row>
     <row r="182" ht="12.75" customHeight="1">
       <c r="A182" s="20"/>
@@ -11715,7 +11527,6 @@
       <c r="BC182" s="20"/>
       <c r="BD182" s="20"/>
       <c r="BE182" s="20"/>
-      <c r="BF182" s="20"/>
     </row>
     <row r="183" ht="12.75" customHeight="1">
       <c r="A183" s="20"/>
@@ -11775,7 +11586,6 @@
       <c r="BC183" s="20"/>
       <c r="BD183" s="20"/>
       <c r="BE183" s="20"/>
-      <c r="BF183" s="20"/>
     </row>
     <row r="184" ht="12.75" customHeight="1">
       <c r="A184" s="20"/>
@@ -11835,7 +11645,6 @@
       <c r="BC184" s="20"/>
       <c r="BD184" s="20"/>
       <c r="BE184" s="20"/>
-      <c r="BF184" s="20"/>
     </row>
     <row r="185" ht="12.75" customHeight="1">
       <c r="A185" s="20"/>
@@ -11895,7 +11704,6 @@
       <c r="BC185" s="20"/>
       <c r="BD185" s="20"/>
       <c r="BE185" s="20"/>
-      <c r="BF185" s="20"/>
     </row>
     <row r="186" ht="12.75" customHeight="1">
       <c r="A186" s="20"/>
@@ -11955,7 +11763,6 @@
       <c r="BC186" s="20"/>
       <c r="BD186" s="20"/>
       <c r="BE186" s="20"/>
-      <c r="BF186" s="20"/>
     </row>
     <row r="187" ht="12.75" customHeight="1">
       <c r="A187" s="20"/>
@@ -12015,7 +11822,6 @@
       <c r="BC187" s="20"/>
       <c r="BD187" s="20"/>
       <c r="BE187" s="20"/>
-      <c r="BF187" s="20"/>
     </row>
     <row r="188" ht="12.75" customHeight="1">
       <c r="A188" s="20"/>
@@ -12075,7 +11881,6 @@
       <c r="BC188" s="20"/>
       <c r="BD188" s="20"/>
       <c r="BE188" s="20"/>
-      <c r="BF188" s="20"/>
     </row>
     <row r="189" ht="12.75" customHeight="1">
       <c r="A189" s="20"/>
@@ -12135,7 +11940,6 @@
       <c r="BC189" s="20"/>
       <c r="BD189" s="20"/>
       <c r="BE189" s="20"/>
-      <c r="BF189" s="20"/>
     </row>
     <row r="190" ht="12.75" customHeight="1">
       <c r="A190" s="20"/>
@@ -12195,7 +11999,6 @@
       <c r="BC190" s="20"/>
       <c r="BD190" s="20"/>
       <c r="BE190" s="20"/>
-      <c r="BF190" s="20"/>
     </row>
     <row r="191" ht="12.75" customHeight="1">
       <c r="A191" s="20"/>
@@ -12255,7 +12058,6 @@
       <c r="BC191" s="20"/>
       <c r="BD191" s="20"/>
       <c r="BE191" s="20"/>
-      <c r="BF191" s="20"/>
     </row>
     <row r="192" ht="12.75" customHeight="1">
       <c r="A192" s="20"/>
@@ -12315,7 +12117,6 @@
       <c r="BC192" s="20"/>
       <c r="BD192" s="20"/>
       <c r="BE192" s="20"/>
-      <c r="BF192" s="20"/>
     </row>
     <row r="193" ht="12.75" customHeight="1">
       <c r="A193" s="20"/>
@@ -12375,7 +12176,6 @@
       <c r="BC193" s="20"/>
       <c r="BD193" s="20"/>
       <c r="BE193" s="20"/>
-      <c r="BF193" s="20"/>
     </row>
     <row r="194" ht="12.75" customHeight="1">
       <c r="A194" s="20"/>
@@ -12435,7 +12235,6 @@
       <c r="BC194" s="20"/>
       <c r="BD194" s="20"/>
       <c r="BE194" s="20"/>
-      <c r="BF194" s="20"/>
     </row>
     <row r="195" ht="12.75" customHeight="1">
       <c r="A195" s="20"/>
@@ -12495,7 +12294,6 @@
       <c r="BC195" s="20"/>
       <c r="BD195" s="20"/>
       <c r="BE195" s="20"/>
-      <c r="BF195" s="20"/>
     </row>
     <row r="196" ht="12.75" customHeight="1">
       <c r="A196" s="20"/>
@@ -12555,7 +12353,6 @@
       <c r="BC196" s="20"/>
       <c r="BD196" s="20"/>
       <c r="BE196" s="20"/>
-      <c r="BF196" s="20"/>
     </row>
     <row r="197" ht="12.75" customHeight="1">
       <c r="A197" s="20"/>
@@ -12615,7 +12412,6 @@
       <c r="BC197" s="20"/>
       <c r="BD197" s="20"/>
       <c r="BE197" s="20"/>
-      <c r="BF197" s="20"/>
     </row>
     <row r="198" ht="12.75" customHeight="1">
       <c r="A198" s="20"/>
@@ -12675,7 +12471,6 @@
       <c r="BC198" s="20"/>
       <c r="BD198" s="20"/>
       <c r="BE198" s="20"/>
-      <c r="BF198" s="20"/>
     </row>
     <row r="199" ht="12.75" customHeight="1">
       <c r="A199" s="20"/>
@@ -12735,7 +12530,6 @@
       <c r="BC199" s="20"/>
       <c r="BD199" s="20"/>
       <c r="BE199" s="20"/>
-      <c r="BF199" s="20"/>
     </row>
     <row r="200" ht="12.75" customHeight="1">
       <c r="A200" s="20"/>
@@ -12795,7 +12589,6 @@
       <c r="BC200" s="20"/>
       <c r="BD200" s="20"/>
       <c r="BE200" s="20"/>
-      <c r="BF200" s="20"/>
     </row>
     <row r="201" ht="12.75" customHeight="1">
       <c r="A201" s="20"/>
@@ -12855,7 +12648,6 @@
       <c r="BC201" s="20"/>
       <c r="BD201" s="20"/>
       <c r="BE201" s="20"/>
-      <c r="BF201" s="20"/>
     </row>
     <row r="202" ht="12.75" customHeight="1">
       <c r="A202" s="20"/>
@@ -12915,7 +12707,6 @@
       <c r="BC202" s="20"/>
       <c r="BD202" s="20"/>
       <c r="BE202" s="20"/>
-      <c r="BF202" s="20"/>
     </row>
     <row r="203" ht="12.75" customHeight="1">
       <c r="A203" s="20"/>
@@ -12975,7 +12766,6 @@
       <c r="BC203" s="20"/>
       <c r="BD203" s="20"/>
       <c r="BE203" s="20"/>
-      <c r="BF203" s="20"/>
     </row>
     <row r="204" ht="12.75" customHeight="1">
       <c r="A204" s="20"/>
@@ -13035,7 +12825,6 @@
       <c r="BC204" s="20"/>
       <c r="BD204" s="20"/>
       <c r="BE204" s="20"/>
-      <c r="BF204" s="20"/>
     </row>
     <row r="205" ht="12.75" customHeight="1">
       <c r="A205" s="20"/>
@@ -13095,7 +12884,6 @@
       <c r="BC205" s="20"/>
       <c r="BD205" s="20"/>
       <c r="BE205" s="20"/>
-      <c r="BF205" s="20"/>
     </row>
     <row r="206" ht="12.75" customHeight="1">
       <c r="A206" s="20"/>
@@ -13155,7 +12943,6 @@
       <c r="BC206" s="20"/>
       <c r="BD206" s="20"/>
       <c r="BE206" s="20"/>
-      <c r="BF206" s="20"/>
     </row>
     <row r="207" ht="12.75" customHeight="1">
       <c r="A207" s="20"/>
@@ -13215,7 +13002,6 @@
       <c r="BC207" s="20"/>
       <c r="BD207" s="20"/>
       <c r="BE207" s="20"/>
-      <c r="BF207" s="20"/>
     </row>
     <row r="208" ht="12.75" customHeight="1">
       <c r="A208" s="20"/>
@@ -13275,7 +13061,6 @@
       <c r="BC208" s="20"/>
       <c r="BD208" s="20"/>
       <c r="BE208" s="20"/>
-      <c r="BF208" s="20"/>
     </row>
     <row r="209" ht="12.75" customHeight="1">
       <c r="A209" s="20"/>
@@ -13335,7 +13120,6 @@
       <c r="BC209" s="20"/>
       <c r="BD209" s="20"/>
       <c r="BE209" s="20"/>
-      <c r="BF209" s="20"/>
     </row>
     <row r="210" ht="12.75" customHeight="1">
       <c r="A210" s="20"/>
@@ -13395,7 +13179,6 @@
       <c r="BC210" s="20"/>
       <c r="BD210" s="20"/>
       <c r="BE210" s="20"/>
-      <c r="BF210" s="20"/>
     </row>
     <row r="211" ht="12.75" customHeight="1">
       <c r="A211" s="20"/>
@@ -13455,7 +13238,6 @@
       <c r="BC211" s="20"/>
       <c r="BD211" s="20"/>
       <c r="BE211" s="20"/>
-      <c r="BF211" s="20"/>
     </row>
     <row r="212" ht="12.75" customHeight="1">
       <c r="A212" s="20"/>
@@ -13515,7 +13297,6 @@
       <c r="BC212" s="20"/>
       <c r="BD212" s="20"/>
       <c r="BE212" s="20"/>
-      <c r="BF212" s="20"/>
     </row>
     <row r="213" ht="12.75" customHeight="1">
       <c r="A213" s="20"/>
@@ -13575,7 +13356,6 @@
       <c r="BC213" s="20"/>
       <c r="BD213" s="20"/>
       <c r="BE213" s="20"/>
-      <c r="BF213" s="20"/>
     </row>
     <row r="214" ht="12.75" customHeight="1">
       <c r="A214" s="20"/>
@@ -13635,7 +13415,6 @@
       <c r="BC214" s="20"/>
       <c r="BD214" s="20"/>
       <c r="BE214" s="20"/>
-      <c r="BF214" s="20"/>
     </row>
     <row r="215" ht="12.75" customHeight="1">
       <c r="A215" s="20"/>
@@ -13695,7 +13474,6 @@
       <c r="BC215" s="20"/>
       <c r="BD215" s="20"/>
       <c r="BE215" s="20"/>
-      <c r="BF215" s="20"/>
     </row>
     <row r="216" ht="12.75" customHeight="1">
       <c r="A216" s="20"/>
@@ -13755,7 +13533,6 @@
       <c r="BC216" s="20"/>
       <c r="BD216" s="20"/>
       <c r="BE216" s="20"/>
-      <c r="BF216" s="20"/>
     </row>
     <row r="217" ht="12.75" customHeight="1">
       <c r="A217" s="20"/>
@@ -13815,7 +13592,6 @@
       <c r="BC217" s="20"/>
       <c r="BD217" s="20"/>
       <c r="BE217" s="20"/>
-      <c r="BF217" s="20"/>
     </row>
     <row r="218" ht="12.75" customHeight="1">
       <c r="A218" s="20"/>
@@ -13875,7 +13651,6 @@
       <c r="BC218" s="20"/>
       <c r="BD218" s="20"/>
       <c r="BE218" s="20"/>
-      <c r="BF218" s="20"/>
     </row>
     <row r="219" ht="12.75" customHeight="1">
       <c r="A219" s="20"/>
@@ -13935,7 +13710,6 @@
       <c r="BC219" s="20"/>
       <c r="BD219" s="20"/>
       <c r="BE219" s="20"/>
-      <c r="BF219" s="20"/>
     </row>
     <row r="220" ht="15.75" customHeight="1"/>
     <row r="221" ht="15.75" customHeight="1"/>
@@ -14717,6 +14491,7 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
APR: updating Excel template to reflect moved column
</commit_message>
<xml_diff>
--- a/core/api/export/templates/APRAnnexI.xlsx
+++ b/core/api/export/templates/APRAnnexI.xlsx
@@ -16,7 +16,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment authorId="0" ref="AT1">
+    <comment authorId="0" ref="AU1">
       <text>
         <t xml:space="preserve">XX meeting, based on the year of the APR and the last ExCom meeting held before the APR. to be derived
 	-Rony Salim Aoun</t>
@@ -164,10 +164,10 @@
     <t xml:space="preserve">Funds advanced (US$) </t>
   </si>
   <si>
-    <t xml:space="preserve">Implementation Delays/Status Report Decisions </t>
+    <t>Date of Completion per Agreements or per Decisions</t>
   </si>
   <si>
-    <t>Date of Completion per Agreements or per Decisions</t>
+    <t xml:space="preserve">Implementation Delays/Status Report Decisions </t>
   </si>
   <si>
     <t xml:space="preserve">Remarks (as of 31 December XXXX) </t>
@@ -254,7 +254,7 @@
       <name val="Times New Roman"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -265,6 +265,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFBFBFBF"/>
         <bgColor rgb="FFBFBFBF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -315,10 +321,10 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="17" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -593,8 +599,8 @@
     <col customWidth="1" min="38" max="38" width="11.25"/>
     <col customWidth="1" min="39" max="43" width="9.25" outlineLevel="1"/>
     <col customWidth="1" min="44" max="45" width="12.13" outlineLevel="1"/>
-    <col customWidth="1" min="46" max="46" width="13.13"/>
-    <col customWidth="1" min="47" max="47" width="12.13"/>
+    <col customWidth="1" min="46" max="46" width="12.13"/>
+    <col customWidth="1" min="47" max="47" width="13.13" outlineLevel="1"/>
     <col customWidth="1" min="48" max="50" width="21.38" outlineLevel="1"/>
     <col customWidth="1" min="51" max="51" width="10.63"/>
     <col customWidth="1" min="52" max="54" width="9.25"/>
@@ -891,10 +897,10 @@
       <c r="AS2" s="17">
         <v>-109351.01</v>
       </c>
-      <c r="AT2" s="18"/>
-      <c r="AU2" s="15">
+      <c r="AT2" s="15">
         <v>39965.0</v>
       </c>
+      <c r="AU2" s="18"/>
       <c r="AV2" s="18"/>
       <c r="AW2" s="18"/>
       <c r="AX2" s="19" t="s">

</xml_diff>

<commit_message>
Removing comments from AnnexI template
</commit_message>
<xml_diff>
--- a/core/api/export/templates/APRAnnexI.xlsx
+++ b/core/api/export/templates/APRAnnexI.xlsx
@@ -10,25 +10,6 @@
   </definedNames>
   <calcPr/>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment authorId="0" ref="A1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	To use the abbreviated value please. Once implemented the comment to be deleted
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3909,10 +3890,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -42755,6 +42732,5 @@
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>